<commit_message>
📊 BIST Screener | 21.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-21.xlsx
+++ b/data/bist_screener_2026-05-21.xlsx
@@ -25946,36 +25946,36 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>61.2</v>
+        <v>14.77</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.1</v>
+        <v>-0.0999</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>45370</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>42630000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>30.01</v>
+        <v>39.14</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.4928</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L588" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
@@ -26018,65 +26018,69 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>79.87</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0306</v>
+        <v>-0.0999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>11370000</v>
+        <v>29500000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>46.55</v>
+        <v>72.91</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
       <c r="I590" s="2" t="inlineStr"/>
       <c r="J590" s="2" t="inlineStr"/>
-      <c r="K590" s="2" t="inlineStr"/>
-      <c r="L590" s="2" t="inlineStr"/>
+      <c r="K590" s="2" t="inlineStr">
+        <is>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L590" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M590" s="2" t="inlineStr"/>
     </row>
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>24.08</v>
+        <v>36.04</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0444</v>
+        <v>-0.0999</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>873490</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>11070000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>32.61</v>
+        <v>52.96</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
       <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="8" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26084,75 +26088,75 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>5.7</v>
+        <v>61.2</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.09089999999999999</v>
+        <v>-0.1</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>24140000</v>
+        <v>45370</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.58</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>46.97</v>
+        <v>30.01</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
+      <c r="I592" s="2" t="inlineStr"/>
       <c r="J592" s="4" t="n">
-        <v>-4.2562</v>
+        <v>0.4928</v>
       </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>36.04</v>
+        <v>123.3</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0999</v>
+        <v>-0.0993</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>11070000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>926710</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>52.96</v>
+        <v>36.39</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26160,21 +26164,21 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>71.65000000000001</v>
+        <v>15.49</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0999</v>
+        <v>-0.09939999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>29500000</v>
+        <v>38910000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>72.91</v>
+        <v>42.3</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26182,12 +26186,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26195,52 +26199,48 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>63.2</v>
+        <v>79.87</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.09710000000000001</v>
+        <v>0.0306</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>147080</v>
+        <v>11370000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>8.550000000000001</v>
+        <v>46.55</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
-      <c r="K595" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
+      <c r="K595" s="6" t="inlineStr"/>
       <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>15.49</v>
+        <v>16.81</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.09939999999999999</v>
+        <v>-0.0839</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>38910000</v>
+        <v>50030000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>42.3</v>
+        <v>28.98</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26248,12 +26248,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26261,21 +26261,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>36.5</v>
+        <v>63.2</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.09710000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>5900000</v>
+        <v>147080</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>37.87</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26283,51 +26283,43 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>60.35</v>
+        <v>2.52</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0607</v>
+        <v>-0.0968</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>718350</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>127640000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>40.42</v>
+        <v>38.61</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
       <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="4" t="n">
-        <v>0.1431</v>
-      </c>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26335,83 +26327,67 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>32.34</v>
+        <v>230.3</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.046</v>
+        <v>-0.0158</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>4900000</v>
+        <v>10060</v>
       </c>
       <c r="E599" s="8" t="n">
-        <v>0.3528</v>
+        <v>0.2578</v>
       </c>
       <c r="F599" s="7" t="n">
-        <v>36.31</v>
-      </c>
-      <c r="G599" s="7" t="n">
-        <v>12.78</v>
-      </c>
+        <v>37.73</v>
+      </c>
+      <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>0.1029</v>
-      </c>
-      <c r="J599" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>123.3</v>
+        <v>167.7</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0993</v>
+        <v>-0.0998</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>926710</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>7580000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>36.39</v>
+        <v>46.94</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26419,58 +26395,62 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>10.04</v>
+        <v>2.17</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.051</v>
+        <v>-0.09960000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>741800</v>
+        <v>19990000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>59.85</v>
+        <v>25.23</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="8" t="n">
-        <v>-23.6291</v>
+        <v>-191.6342</v>
       </c>
       <c r="J601" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-0.8093</v>
       </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>167.7</v>
+        <v>36.5</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0998</v>
+        <v>-0.0925</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>7580000</v>
+        <v>5900000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>46.94</v>
+        <v>37.87</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26478,12 +26458,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26491,21 +26471,21 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>14.77</v>
+        <v>12.7</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0999</v>
+        <v>-0.0593</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>42630000</v>
+        <v>27420000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>39.14</v>
+        <v>37.39</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26513,12 +26493,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26526,21 +26506,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>26.6</v>
+        <v>5.89</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.07190000000000001</v>
+        <v>-0.02</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>19960000</v>
+        <v>8420000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>46.76</v>
+        <v>29.99</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26548,53 +26528,47 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.17</v>
+        <v>60.35</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.09960000000000001</v>
+        <v>-0.0607</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>19990000</v>
+        <v>718350</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>1</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>25.23</v>
+        <v>40.42</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.1431</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26602,21 +26576,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>2.52</v>
+        <v>163</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0968</v>
+        <v>-0.08119999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>127640000</v>
+        <v>7570000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>38.61</v>
+        <v>31.96</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26624,12 +26598,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26637,21 +26611,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>12.7</v>
+        <v>26.6</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0593</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>27420000</v>
+        <v>19960000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>37.39</v>
+        <v>46.76</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26659,12 +26633,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26672,57 +26646,71 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>5.89</v>
+        <v>24.08</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.02</v>
+        <v>-0.0444</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>8420000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>873490</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.9698</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>29.99</v>
+        <v>32.61</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="J608" s="4" t="n">
+        <v>0.6453</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>16.81</v>
+        <v>5.7</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0839</v>
+        <v>-0.09089999999999999</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>50030000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>24140000</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>28.98</v>
+        <v>46.97</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26730,7 +26718,7 @@
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26738,34 +26726,42 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>163</v>
+        <v>32.34</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.08119999999999999</v>
+        <v>-0.046</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>7570000</v>
-      </c>
-      <c r="E610" s="2" t="inlineStr"/>
+        <v>4900000</v>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F610" s="3" t="n">
-        <v>31.96</v>
-      </c>
-      <c r="G610" s="2" t="inlineStr"/>
+        <v>36.31</v>
+      </c>
+      <c r="G610" s="3" t="n">
+        <v>12.78</v>
+      </c>
       <c r="H610" s="2" t="inlineStr"/>
-      <c r="I610" s="2" t="inlineStr"/>
-      <c r="J610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J610" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26773,28 +26769,32 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>230.3</v>
+        <v>10.04</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.0158</v>
+        <v>-0.051</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>10060</v>
+        <v>741800</v>
       </c>
       <c r="E611" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.95</v>
       </c>
       <c r="F611" s="7" t="n">
-        <v>37.73</v>
+        <v>59.85</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
@@ -26825,7 +26825,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>21.05.2026 15:30</t>
+          <t>21.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 21.05.2026 17:37 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-21.xlsx
+++ b/data/bist_screener_2026-05-21.xlsx
@@ -25946,34 +25946,40 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>14.77</v>
+        <v>2.17</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0999</v>
+        <v>-0.09960000000000001</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>42630000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>19990000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>39.14</v>
+        <v>25.23</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25981,23 +25987,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>30</v>
+        <v>16.81</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0046</v>
+        <v>-0.0839</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>19660000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>50030000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>49.99</v>
+        <v>28.98</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26005,12 +26009,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26018,21 +26022,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>71.65000000000001</v>
+        <v>14.77</v>
       </c>
       <c r="C590" s="4" t="n">
         <v>-0.0999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>29500000</v>
+        <v>42630000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>72.91</v>
+        <v>39.14</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26040,12 +26044,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26053,21 +26057,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>36.04</v>
+        <v>163</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0999</v>
+        <v>-0.08119999999999999</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>11070000</v>
+        <v>7570000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>52.96</v>
+        <v>31.96</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26075,12 +26079,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26088,75 +26092,79 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>61.2</v>
+        <v>5.7</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.1</v>
+        <v>-0.09089999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>45370</v>
+        <v>24140000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.58</v>
+        <v>0.1672</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>30.01</v>
+        <v>46.97</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
       <c r="J592" s="4" t="n">
-        <v>0.4928</v>
+        <v>-4.2562</v>
       </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>VKING</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>123.3</v>
+        <v>24.08</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0993</v>
+        <v>-0.0444</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>926710</v>
+        <v>873490</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.9698</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>36.39</v>
+        <v>32.61</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="8" t="n">
-        <v>-0.4897</v>
+        <v>0.6453</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26164,34 +26172,40 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>15.49</v>
+        <v>123.3</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.09939999999999999</v>
+        <v>-0.0993</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>38910000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>926710</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>42.3</v>
+        <v>36.39</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26199,48 +26213,56 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>79.87</v>
+        <v>2.52</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0306</v>
+        <v>-0.0968</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>11370000</v>
+        <v>127640000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>46.55</v>
+        <v>38.61</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="6" t="inlineStr"/>
-      <c r="K595" s="6" t="inlineStr"/>
-      <c r="L595" s="6" t="inlineStr"/>
+      <c r="K595" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>16.81</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0839</v>
+        <v>-0.0999</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>50030000</v>
+        <v>29500000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>28.98</v>
+        <v>72.91</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26248,12 +26270,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26261,21 +26283,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>63.2</v>
+        <v>26.6</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.09710000000000001</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>147080</v>
+        <v>19960000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>8.550000000000001</v>
+        <v>46.76</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26283,43 +26305,55 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>2.52</v>
+        <v>32.34</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0968</v>
+        <v>-0.046</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>127640000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>4900000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>38.61</v>
-      </c>
-      <c r="G598" s="2" t="inlineStr"/>
+        <v>36.31</v>
+      </c>
+      <c r="G598" s="3" t="n">
+        <v>12.78</v>
+      </c>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>0.1029</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26327,23 +26361,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>230.3</v>
+        <v>15.49</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0158</v>
+        <v>-0.09939999999999999</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>10060</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>38910000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>37.73</v>
+        <v>42.3</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26351,30 +26383,34 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>167.7</v>
+        <v>12.7</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.0998</v>
+        <v>-0.0593</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>7580000</v>
+        <v>27420000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>46.94</v>
+        <v>37.39</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26382,12 +26418,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26395,40 +26431,36 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>2.17</v>
+        <v>30</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.09960000000000001</v>
+        <v>-0.0046</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>19990000</v>
+        <v>19660000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>1</v>
+        <v>0.2667</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>25.23</v>
+        <v>49.99</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26436,21 +26468,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>36.5</v>
+        <v>63.2</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0925</v>
+        <v>-0.09710000000000001</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>5900000</v>
+        <v>147080</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>37.87</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26458,34 +26490,30 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>12.7</v>
+        <v>5.89</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0593</v>
+        <v>-0.02</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>27420000</v>
+        <v>8420000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>37.39</v>
+        <v>29.99</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26493,34 +26521,30 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>5.89</v>
+        <v>167.7</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.02</v>
+        <v>-0.0998</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>8420000</v>
+        <v>7580000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>29.99</v>
+        <v>46.94</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26528,69 +26552,63 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>60.35</v>
+        <v>79.87</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>-0.0607</v>
+        <v>0.0306</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>718350</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>11370000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>40.42</v>
+        <v>46.55</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="8" t="n">
-        <v>0.1431</v>
-      </c>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="J605" s="6" t="inlineStr"/>
+      <c r="K605" s="6" t="inlineStr"/>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>163</v>
+        <v>230.3</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.08119999999999999</v>
+        <v>-0.0158</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>7570000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>10060</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>31.96</v>
+        <v>37.73</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26598,86 +26616,78 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>26.6</v>
+        <v>61.2</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.07190000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>19960000</v>
-      </c>
-      <c r="E607" s="6" t="inlineStr"/>
+        <v>45370</v>
+      </c>
+      <c r="E607" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F607" s="7" t="n">
-        <v>46.76</v>
+        <v>30.01</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="6" t="inlineStr"/>
-      <c r="J607" s="6" t="inlineStr"/>
+      <c r="J607" s="8" t="n">
+        <v>0.4928</v>
+      </c>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VKING</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>24.08</v>
+        <v>36.04</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>-0.0444</v>
+        <v>-0.0999</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>873490</v>
-      </c>
-      <c r="E608" s="4" t="n">
-        <v>0.9698</v>
-      </c>
+        <v>11070000</v>
+      </c>
+      <c r="E608" s="2" t="inlineStr"/>
       <c r="F608" s="3" t="n">
-        <v>32.61</v>
+        <v>52.96</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
       <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="4" t="n">
-        <v>0.6453</v>
-      </c>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L608" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST ORMAN KAĞIT BASIM, BIST ANA, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M608" s="2" t="inlineStr"/>
@@ -26685,40 +26695,38 @@
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>5.7</v>
+        <v>60.35</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.09089999999999999</v>
+        <v>-0.0607</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>24140000</v>
+        <v>718350</v>
       </c>
       <c r="E609" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F609" s="7" t="n">
-        <v>46.97</v>
+        <v>40.42</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
+      <c r="I609" s="6" t="inlineStr"/>
       <c r="J609" s="8" t="n">
-        <v>-4.2562</v>
+        <v>0.1431</v>
       </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26726,81 +26734,73 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>32.34</v>
+        <v>10.04</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.046</v>
+        <v>-0.051</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>4900000</v>
+        <v>741800</v>
       </c>
       <c r="E610" s="4" t="n">
-        <v>0.3528</v>
+        <v>0.95</v>
       </c>
       <c r="F610" s="3" t="n">
-        <v>36.31</v>
-      </c>
-      <c r="G610" s="3" t="n">
-        <v>12.78</v>
-      </c>
+        <v>59.85</v>
+      </c>
+      <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
       <c r="I610" s="4" t="n">
-        <v>0.1029</v>
+        <v>-23.6291</v>
       </c>
       <c r="J610" s="4" t="n">
-        <v>-1.4864</v>
+        <v>-0.4678</v>
       </c>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L610" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L610" s="2" t="inlineStr"/>
       <c r="M610" s="2" t="inlineStr"/>
     </row>
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>10.04</v>
+        <v>36.5</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.051</v>
+        <v>-0.0925</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>741800</v>
-      </c>
-      <c r="E611" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>5900000</v>
+      </c>
+      <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>59.85</v>
+        <v>37.87</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J611" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26825,7 +26825,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>21.05.2026 16:30</t>
+          <t>21.05.2026 17:37</t>
         </is>
       </c>
     </row>

</xml_diff>